<commit_message>
ajout JDV J407 et J405 a67e5d8db838da4d95731b5ed1a63dc64d26b18a
</commit_message>
<xml_diff>
--- a/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-consent-accord.xlsx
+++ b/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-consent-accord.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2208" uniqueCount="371">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2209" uniqueCount="372">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-17T10:53:05+00:00</t>
+    <t>2026-06-03T14:26:22+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -468,10 +468,14 @@
 </t>
   </si>
   <si>
-    <t>Optional Extensions Element</t>
-  </si>
-  <si>
-    <t>Optional Extension Element - found in all resources.</t>
+    <t>R5: Effective period for this Consent (new)</t>
+  </si>
+  <si>
+    <t>R5: `Consent.period` (new:Period)</t>
+  </si>
+  <si>
+    <t>Element `Consent.period` has a context of Consent based on following the parent source element upwards and mapping to `Consent`.
+Element `Consent.period` has no mapping targets in FHIR R4. Typically, this is because the element has been added (is a new element).</t>
   </si>
   <si>
     <t xml:space="preserve">ele-1
@@ -2606,7 +2610,9 @@
       <c r="M10" t="s" s="2">
         <v>147</v>
       </c>
-      <c r="N10" s="2"/>
+      <c r="N10" t="s" s="2">
+        <v>148</v>
+      </c>
       <c r="O10" s="2"/>
       <c r="P10" t="s" s="2">
         <v>78</v>
@@ -2664,13 +2670,13 @@
         <v>80</v>
       </c>
       <c r="AI10" t="s" s="2">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="AJ10" t="s" s="2">
         <v>142</v>
       </c>
       <c r="AK10" t="s" s="2">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="AL10" t="s" s="2">
         <v>78</v>
@@ -2679,7 +2685,7 @@
         <v>78</v>
       </c>
       <c r="AN10" t="s" s="2">
-        <v>134</v>
+        <v>78</v>
       </c>
       <c r="AO10" t="s" s="2">
         <v>78</v>
@@ -2687,14 +2693,14 @@
     </row>
     <row r="11">
       <c r="A11" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
@@ -2716,16 +2722,16 @@
         <v>136</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="N11" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O11" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P11" t="s" s="2">
         <v>78</v>
@@ -2774,7 +2780,7 @@
         <v>78</v>
       </c>
       <c r="AF11" t="s" s="2">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="AG11" t="s" s="2">
         <v>79</v>
@@ -2806,10 +2812,10 @@
     </row>
     <row r="12">
       <c r="A12" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B12" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" t="s" s="2">
@@ -2832,16 +2838,16 @@
         <v>92</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="N12" t="s" s="2">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="O12" s="2"/>
       <c r="P12" t="s" s="2">
@@ -2855,7 +2861,7 @@
         <v>78</v>
       </c>
       <c r="T12" t="s" s="2">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="U12" t="s" s="2">
         <v>78</v>
@@ -2891,7 +2897,7 @@
         <v>78</v>
       </c>
       <c r="AF12" t="s" s="2">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="AG12" t="s" s="2">
         <v>79</v>
@@ -2909,24 +2915,24 @@
         <v>78</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="AM12" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN12" t="s" s="2">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="AO12" t="s" s="2">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" t="s" s="2">
@@ -2952,16 +2958,16 @@
         <v>111</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="N13" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="O13" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="P13" t="s" s="2">
         <v>78</v>
@@ -2986,13 +2992,13 @@
         <v>78</v>
       </c>
       <c r="X13" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Y13" t="s" s="2">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="Z13" t="s" s="2">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="AA13" t="s" s="2">
         <v>78</v>
@@ -3010,7 +3016,7 @@
         <v>78</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>91</v>
@@ -3028,24 +3034,24 @@
         <v>78</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="AM13" t="s" s="2">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="AN13" t="s" s="2">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="AO13" t="s" s="2">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -3068,13 +3074,13 @@
         <v>92</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -3101,13 +3107,13 @@
         <v>78</v>
       </c>
       <c r="X14" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Y14" t="s" s="2">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="Z14" t="s" s="2">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="AA14" t="s" s="2">
         <v>78</v>
@@ -3125,7 +3131,7 @@
         <v>78</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>91</v>
@@ -3157,10 +3163,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -3183,13 +3189,13 @@
         <v>92</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -3216,13 +3222,13 @@
         <v>78</v>
       </c>
       <c r="X15" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Y15" t="s" s="2">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="Z15" t="s" s="2">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="AA15" t="s" s="2">
         <v>78</v>
@@ -3240,7 +3246,7 @@
         <v>78</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>91</v>
@@ -3258,24 +3264,24 @@
         <v>78</v>
       </c>
       <c r="AL15" t="s" s="2">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="AM15" t="s" s="2">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="AN15" t="s" s="2">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="AO15" t="s" s="2">
-        <v>193</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3298,16 +3304,16 @@
         <v>92</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="N16" t="s" s="2">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O16" s="2"/>
       <c r="P16" t="s" s="2">
@@ -3357,7 +3363,7 @@
         <v>78</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>79</v>
@@ -3375,24 +3381,24 @@
         <v>78</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="AM16" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AN16" t="s" s="2">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="AO16" t="s" s="2">
-        <v>201</v>
+        <v>202</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3415,16 +3421,16 @@
         <v>92</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="O17" s="2"/>
       <c r="P17" t="s" s="2">
@@ -3474,7 +3480,7 @@
         <v>78</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>79</v>
@@ -3489,31 +3495,31 @@
         <v>103</v>
       </c>
       <c r="AK17" t="s" s="2">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="AL17" t="s" s="2">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="AM17" t="s" s="2">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="AN17" t="s" s="2">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="AO17" t="s" s="2">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
@@ -3532,16 +3538,16 @@
         <v>92</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
@@ -3591,7 +3597,7 @@
         <v>78</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>79</v>
@@ -3606,31 +3612,31 @@
         <v>103</v>
       </c>
       <c r="AK18" t="s" s="2">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AM18" t="s" s="2">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="AN18" t="s" s="2">
         <v>78</v>
       </c>
       <c r="AO18" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="E19" s="2"/>
       <c r="F19" t="s" s="2">
@@ -3649,13 +3655,13 @@
         <v>92</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="N19" s="2"/>
       <c r="O19" s="2"/>
@@ -3706,7 +3712,7 @@
         <v>78</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>79</v>
@@ -3724,7 +3730,7 @@
         <v>78</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="AM19" t="s" s="2">
         <v>78</v>
@@ -3733,15 +3739,15 @@
         <v>78</v>
       </c>
       <c r="AO19" t="s" s="2">
-        <v>227</v>
+        <v>228</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3764,16 +3770,16 @@
         <v>92</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="N20" t="s" s="2">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
@@ -3823,7 +3829,7 @@
         <v>78</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>79</v>
@@ -3844,7 +3850,7 @@
         <v>78</v>
       </c>
       <c r="AM20" t="s" s="2">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="AN20" t="s" s="2">
         <v>78</v>
@@ -3855,10 +3861,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -3881,13 +3887,13 @@
         <v>78</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3938,7 +3944,7 @@
         <v>78</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>79</v>
@@ -3970,10 +3976,10 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
@@ -3996,13 +4002,13 @@
         <v>78</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -4053,7 +4059,7 @@
         <v>78</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>79</v>
@@ -4077,7 +4083,7 @@
         <v>78</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AO22" t="s" s="2">
         <v>78</v>
@@ -4085,14 +4091,14 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
@@ -4114,13 +4120,13 @@
         <v>136</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -4170,7 +4176,7 @@
         <v>78</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>79</v>
@@ -4194,7 +4200,7 @@
         <v>78</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AO23" t="s" s="2">
         <v>78</v>
@@ -4202,14 +4208,14 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" t="s" s="2">
@@ -4231,16 +4237,16 @@
         <v>136</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O24" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>78</v>
@@ -4289,7 +4295,7 @@
         <v>78</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>79</v>
@@ -4321,10 +4327,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -4350,10 +4356,10 @@
         <v>105</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -4404,7 +4410,7 @@
         <v>78</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>79</v>
@@ -4413,7 +4419,7 @@
         <v>91</v>
       </c>
       <c r="AI25" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AJ25" t="s" s="2">
         <v>103</v>
@@ -4436,10 +4442,10 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
@@ -4465,13 +4471,13 @@
         <v>105</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
@@ -4521,7 +4527,7 @@
         <v>78</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>79</v>
@@ -4530,7 +4536,7 @@
         <v>91</v>
       </c>
       <c r="AI26" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AJ26" t="s" s="2">
         <v>103</v>
@@ -4553,10 +4559,10 @@
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -4579,19 +4585,19 @@
         <v>92</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="O27" t="s" s="2">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>78</v>
@@ -4616,13 +4622,13 @@
         <v>78</v>
       </c>
       <c r="X27" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Y27" t="s" s="2">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="Z27" t="s" s="2">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="AA27" t="s" s="2">
         <v>78</v>
@@ -4640,7 +4646,7 @@
         <v>78</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>79</v>
@@ -4649,7 +4655,7 @@
         <v>91</v>
       </c>
       <c r="AI27" t="s" s="2">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="AJ27" t="s" s="2">
         <v>103</v>
@@ -4672,10 +4678,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -4698,13 +4704,13 @@
         <v>92</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -4755,7 +4761,7 @@
         <v>78</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>79</v>
@@ -4787,10 +4793,10 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4813,13 +4819,13 @@
         <v>78</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N29" s="2"/>
       <c r="O29" s="2"/>
@@ -4870,7 +4876,7 @@
         <v>78</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>79</v>
@@ -4894,7 +4900,7 @@
         <v>78</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AO29" t="s" s="2">
         <v>78</v>
@@ -4902,14 +4908,14 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
@@ -4931,13 +4937,13 @@
         <v>136</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O30" s="2"/>
       <c r="P30" t="s" s="2">
@@ -4987,7 +4993,7 @@
         <v>78</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>79</v>
@@ -5011,7 +5017,7 @@
         <v>78</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AO30" t="s" s="2">
         <v>78</v>
@@ -5019,14 +5025,14 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -5048,16 +5054,16 @@
         <v>136</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O31" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P31" t="s" s="2">
         <v>78</v>
@@ -5106,7 +5112,7 @@
         <v>78</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>79</v>
@@ -5138,10 +5144,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5164,13 +5170,13 @@
         <v>92</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="N32" s="2"/>
       <c r="O32" s="2"/>
@@ -5221,7 +5227,7 @@
         <v>78</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>91</v>
@@ -5253,10 +5259,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5279,13 +5285,13 @@
         <v>78</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" s="2"/>
@@ -5336,7 +5342,7 @@
         <v>78</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>79</v>
@@ -5368,10 +5374,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -5394,13 +5400,13 @@
         <v>78</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="N34" s="2"/>
       <c r="O34" s="2"/>
@@ -5451,7 +5457,7 @@
         <v>78</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>79</v>
@@ -5483,10 +5489,10 @@
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -5509,13 +5515,13 @@
         <v>92</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>286</v>
+        <v>287</v>
       </c>
       <c r="N35" s="2"/>
       <c r="O35" s="2"/>
@@ -5566,7 +5572,7 @@
         <v>78</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>79</v>
@@ -5598,10 +5604,10 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
@@ -5624,13 +5630,13 @@
         <v>78</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N36" s="2"/>
       <c r="O36" s="2"/>
@@ -5681,7 +5687,7 @@
         <v>78</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>79</v>
@@ -5705,7 +5711,7 @@
         <v>78</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AO36" t="s" s="2">
         <v>78</v>
@@ -5713,14 +5719,14 @@
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" t="s" s="2">
@@ -5742,13 +5748,13 @@
         <v>136</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O37" s="2"/>
       <c r="P37" t="s" s="2">
@@ -5798,7 +5804,7 @@
         <v>78</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>79</v>
@@ -5822,7 +5828,7 @@
         <v>78</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AO37" t="s" s="2">
         <v>78</v>
@@ -5830,14 +5836,14 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E38" s="2"/>
       <c r="F38" t="s" s="2">
@@ -5859,16 +5865,16 @@
         <v>136</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O38" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P38" t="s" s="2">
         <v>78</v>
@@ -5917,7 +5923,7 @@
         <v>78</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>79</v>
@@ -5949,10 +5955,10 @@
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -5978,10 +5984,10 @@
         <v>111</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="N39" s="2"/>
       <c r="O39" s="2"/>
@@ -6008,13 +6014,13 @@
         <v>78</v>
       </c>
       <c r="X39" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Y39" t="s" s="2">
-        <v>293</v>
+        <v>294</v>
       </c>
       <c r="Z39" t="s" s="2">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="AA39" t="s" s="2">
         <v>78</v>
@@ -6032,7 +6038,7 @@
         <v>78</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>79</v>
@@ -6064,10 +6070,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6090,13 +6096,13 @@
         <v>92</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="N40" s="2"/>
       <c r="O40" s="2"/>
@@ -6147,7 +6153,7 @@
         <v>78</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>79</v>
@@ -6179,10 +6185,10 @@
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6205,13 +6211,13 @@
         <v>78</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="N41" s="2"/>
       <c r="O41" s="2"/>
@@ -6219,7 +6225,7 @@
         <v>78</v>
       </c>
       <c r="Q41" t="s" s="2">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="R41" t="s" s="2">
         <v>78</v>
@@ -6264,7 +6270,7 @@
         <v>78</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>79</v>
@@ -6296,10 +6302,10 @@
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>303</v>
+        <v>304</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -6322,13 +6328,13 @@
         <v>78</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N42" s="2"/>
       <c r="O42" s="2"/>
@@ -6379,7 +6385,7 @@
         <v>78</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>79</v>
@@ -6403,7 +6409,7 @@
         <v>78</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AO42" t="s" s="2">
         <v>78</v>
@@ -6411,14 +6417,14 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
@@ -6440,13 +6446,13 @@
         <v>136</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="N43" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
@@ -6496,7 +6502,7 @@
         <v>78</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>79</v>
@@ -6520,7 +6526,7 @@
         <v>78</v>
       </c>
       <c r="AN43" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AO43" t="s" s="2">
         <v>78</v>
@@ -6528,14 +6534,14 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -6557,16 +6563,16 @@
         <v>136</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="N44" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O44" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P44" t="s" s="2">
         <v>78</v>
@@ -6615,7 +6621,7 @@
         <v>78</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>79</v>
@@ -6647,10 +6653,10 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
@@ -6673,13 +6679,13 @@
         <v>78</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>308</v>
+        <v>309</v>
       </c>
       <c r="N45" s="2"/>
       <c r="O45" s="2"/>
@@ -6706,13 +6712,13 @@
         <v>78</v>
       </c>
       <c r="X45" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Y45" t="s" s="2">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="Z45" t="s" s="2">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="AA45" t="s" s="2">
         <v>78</v>
@@ -6730,7 +6736,7 @@
         <v>78</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>91</v>
@@ -6762,10 +6768,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -6788,13 +6794,13 @@
         <v>78</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>312</v>
+        <v>313</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -6845,7 +6851,7 @@
         <v>78</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>91</v>
@@ -6877,10 +6883,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -6903,23 +6909,23 @@
         <v>92</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="N47" t="s" s="2">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
         <v>78</v>
       </c>
       <c r="Q47" t="s" s="2">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="R47" t="s" s="2">
         <v>78</v>
@@ -6940,13 +6946,13 @@
         <v>78</v>
       </c>
       <c r="X47" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="Y47" t="s" s="2">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Z47" t="s" s="2">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="AA47" t="s" s="2">
         <v>78</v>
@@ -6964,7 +6970,7 @@
         <v>78</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>79</v>
@@ -6996,10 +7002,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7022,16 +7028,16 @@
         <v>92</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="N48" t="s" s="2">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="O48" s="2"/>
       <c r="P48" t="s" s="2">
@@ -7057,13 +7063,13 @@
         <v>78</v>
       </c>
       <c r="X48" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Y48" t="s" s="2">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="Z48" t="s" s="2">
-        <v>329</v>
+        <v>330</v>
       </c>
       <c r="AA48" t="s" s="2">
         <v>78</v>
@@ -7081,7 +7087,7 @@
         <v>78</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>323</v>
+        <v>324</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>79</v>
@@ -7113,10 +7119,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7139,16 +7145,16 @@
         <v>92</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="N49" t="s" s="2">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="O49" s="2"/>
       <c r="P49" t="s" s="2">
@@ -7174,13 +7180,13 @@
         <v>78</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Y49" t="s" s="2">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="Z49" t="s" s="2">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>78</v>
@@ -7198,7 +7204,7 @@
         <v>78</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>79</v>
@@ -7230,10 +7236,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -7256,16 +7262,16 @@
         <v>92</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="N50" t="s" s="2">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="O50" s="2"/>
       <c r="P50" t="s" s="2">
@@ -7291,13 +7297,13 @@
         <v>78</v>
       </c>
       <c r="X50" t="s" s="2">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Y50" t="s" s="2">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="Z50" t="s" s="2">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="AA50" t="s" s="2">
         <v>78</v>
@@ -7315,7 +7321,7 @@
         <v>78</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>336</v>
+        <v>337</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>79</v>
@@ -7347,10 +7353,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -7373,16 +7379,16 @@
         <v>92</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="N51" t="s" s="2">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
@@ -7408,13 +7414,13 @@
         <v>78</v>
       </c>
       <c r="X51" t="s" s="2">
-        <v>320</v>
+        <v>321</v>
       </c>
       <c r="Y51" t="s" s="2">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="Z51" t="s" s="2">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="AA51" t="s" s="2">
         <v>78</v>
@@ -7432,7 +7438,7 @@
         <v>78</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>79</v>
@@ -7464,10 +7470,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -7490,16 +7496,16 @@
         <v>92</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
@@ -7549,7 +7555,7 @@
         <v>78</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>79</v>
@@ -7581,10 +7587,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -7607,13 +7613,13 @@
         <v>92</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="N53" s="2"/>
       <c r="O53" s="2"/>
@@ -7621,7 +7627,7 @@
         <v>78</v>
       </c>
       <c r="Q53" t="s" s="2">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="R53" t="s" s="2">
         <v>78</v>
@@ -7666,7 +7672,7 @@
         <v>78</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>79</v>
@@ -7690,7 +7696,7 @@
         <v>78</v>
       </c>
       <c r="AN53" t="s" s="2">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="AO53" t="s" s="2">
         <v>78</v>
@@ -7698,10 +7704,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -7724,13 +7730,13 @@
         <v>78</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="N54" s="2"/>
       <c r="O54" s="2"/>
@@ -7781,7 +7787,7 @@
         <v>78</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>79</v>
@@ -7805,7 +7811,7 @@
         <v>78</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AO54" t="s" s="2">
         <v>78</v>
@@ -7813,14 +7819,14 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" t="s" s="2">
@@ -7842,13 +7848,13 @@
         <v>136</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="N55" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
@@ -7898,7 +7904,7 @@
         <v>78</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>79</v>
@@ -7922,7 +7928,7 @@
         <v>78</v>
       </c>
       <c r="AN55" t="s" s="2">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="AO55" t="s" s="2">
         <v>78</v>
@@ -7930,14 +7936,14 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>358</v>
+        <v>359</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" t="s" s="2">
@@ -7959,16 +7965,16 @@
         <v>136</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="N56" t="s" s="2">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="O56" t="s" s="2">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="P56" t="s" s="2">
         <v>78</v>
@@ -8017,7 +8023,7 @@
         <v>78</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>79</v>
@@ -8049,10 +8055,10 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
@@ -8078,10 +8084,10 @@
         <v>111</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>361</v>
+        <v>362</v>
       </c>
       <c r="N57" s="2"/>
       <c r="O57" s="2"/>
@@ -8108,13 +8114,13 @@
         <v>78</v>
       </c>
       <c r="X57" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Y57" t="s" s="2">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="Z57" t="s" s="2">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="AA57" t="s" s="2">
         <v>78</v>
@@ -8132,7 +8138,7 @@
         <v>78</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>91</v>
@@ -8164,10 +8170,10 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -8190,13 +8196,13 @@
         <v>92</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="N58" s="2"/>
       <c r="O58" s="2"/>
@@ -8247,7 +8253,7 @@
         <v>78</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>91</v>
@@ -8279,10 +8285,10 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -8308,10 +8314,10 @@
         <v>81</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>369</v>
+        <v>370</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="N59" s="2"/>
       <c r="O59" s="2"/>
@@ -8362,7 +8368,7 @@
         <v>78</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>79</v>

</xml_diff>